<commit_message>
Real 2026 team names: Bison Boys and Frombys
Auston Chen's team becomes Bison Boys, Mike Grosh's becomes Frombys.
Starz & Scrubz unchanged. Team ids are untouched, so nothing already
scored is affected.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CGpnJVRovZyqcFpNbHcPa8
</commit_message>
<xml_diff>
--- a/cms/SycamoreCup-CMS.xlsx
+++ b/cms/SycamoreCup-CMS.xlsx
@@ -2404,7 +2404,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Team One</t>
+          <t>Bison Boys</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Team One</t>
+          <t>Bison Boys</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Team One</t>
+          <t>Bison Boys</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Team One</t>
+          <t>Bison Boys</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Team Two</t>
+          <t>Frombys</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Team Two</t>
+          <t>Frombys</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Team Two</t>
+          <t>Frombys</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Team Two</t>
+          <t>Frombys</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Team Three</t>
+          <t>Starz &amp; Scrubz</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Team Three</t>
+          <t>Starz &amp; Scrubz</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Team Three</t>
+          <t>Starz &amp; Scrubz</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Team Three</t>
+          <t>Starz &amp; Scrubz</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -10134,7 +10134,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sign-in sheet is closable; Justin Quinn's fun facts added
"Who's playing?" could only be dismissed by tapping the backdrop, and only once
you had already claimed a card — so anyone who just wanted to watch the scores
was trapped behind it. It now has an X in the corner, closes on backdrop tap and
on Escape, and the X carries an inline handler so it still works if the module
never executes (the Firebase import can stall on a weak signal).

Justin's 16 answers went into the CMS FunFacts tab and funFactsByPlayer was
regenerated from the sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CGpnJVRovZyqcFpNbHcPa8
</commit_message>
<xml_diff>
--- a/cms/SycamoreCup-CMS.xlsx
+++ b/cms/SycamoreCup-CMS.xlsx
@@ -2745,7 +2745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E232"/>
+  <dimension ref="A1:E248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8554,6 +8554,406 @@
       <c r="E232" t="inlineStr">
         <is>
           <t>Pineapple Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>golfer</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Tiger</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>sportsTeam</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Florida Gators</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>athlete</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>MJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>comedian</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Eddie Murphy</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>actress</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Natalie Portman</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>jersey</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>80s Bulls jersey with script Chicago</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>chip</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Nachos Cheese Doritos</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>candy</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Reese's</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>golfClub</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>8i</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>distanceShot</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>150yds</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>album</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>August and Everything After by the Counting Crows</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>dish</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Chicken Parm</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>star</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Abella Danger</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>warMovie</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Does Braveheart count? If not, Inglourious Basterds</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>sportsMovie</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Friday Night Lights</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>justin-quinn</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Justin Quinn</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>comedyMovie</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Wedding Crashers</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rob Vassallo's 2023-set fun facts — his card is complete at 16
No overlap with the 2024 answers already on file, so nothing was overwritten.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CGpnJVRovZyqcFpNbHcPa8
</commit_message>
<xml_diff>
--- a/cms/SycamoreCup-CMS.xlsx
+++ b/cms/SycamoreCup-CMS.xlsx
@@ -2745,7 +2745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E248"/>
+  <dimension ref="A1:E256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8954,6 +8954,206 @@
       <c r="E248" t="inlineStr">
         <is>
           <t>Wedding Crashers</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>rob-vassallo</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Rob Vassallo</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>golfer</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>John Daly</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>rob-vassallo</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Rob Vassallo</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>sportsTeam</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>GO BIRDS, DICKHEAD!</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>rob-vassallo</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Rob Vassallo</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>athlete</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Allen Iverson</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>rob-vassallo</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Rob Vassallo</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>comedian</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Myself</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>rob-vassallo</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Rob Vassallo</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>actress</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Sloan from Entourage</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>rob-vassallo</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Rob Vassallo</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>jersey</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Chase Utley</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>rob-vassallo</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Rob Vassallo</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>chip</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Jalapeño Kettle Chips</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>rob-vassallo</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Rob Vassallo</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>candy</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Reese’s Fastbreak</t>
         </is>
       </c>
     </row>

</xml_diff>